<commit_message>
Minor modifications, including bug fixed for names on alluvial plots
</commit_message>
<xml_diff>
--- a/data/Curation_data/manual_curation.xlsx
+++ b/data/Curation_data/manual_curation.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GITHUB_REPO\biogps_essoils\data\Curation_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0E9411C-48F2-4297-B305-87CA16EC5A0D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CEC0FAB-A3AA-4778-AF9A-E11138EE7526}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="17256" windowHeight="5316" activeTab="1" xr2:uid="{B08FDB75-03EE-42FB-9439-6A55BCF9F065}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="17256" windowHeight="5316" activeTab="6" xr2:uid="{B08FDB75-03EE-42FB-9439-6A55BCF9F065}"/>
   </bookViews>
   <sheets>
     <sheet name="multiple_genes" sheetId="1" r:id="rId1"/>
@@ -24447,6 +24447,8 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="20.77734375" customWidth="1"/>
+    <col min="4" max="4" width="18" customWidth="1"/>
+    <col min="6" max="6" width="99.33203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">

</xml_diff>